<commit_message>
N2 PCO con la estructura de MP: 4 pasos, prompt limpio y loop por caso (Nómina, Compensación, Selección, Talento); grupos mezclados con caso; datasets PCO sin respuestas en el LÉAME
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datasets/pco/01 Estudio salarial sintético.xlsx
+++ b/datasets/pco/01 Estudio salarial sintético.xlsx
@@ -1159,7 +1159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -1207,13 +1207,6 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Trampas a propósito: la familia Tecnología paga más en mercado; hay cargos con alta rotación y salario bajo el P25.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>